<commit_message>
correction of wrongly sorted files and correction of wong calculation yield to more than 100 % yield in some cases
</commit_message>
<xml_diff>
--- a/experimental_data/irradiations/additives/bases_screening/na2co3_yield.xlsx
+++ b/experimental_data/irradiations/additives/bases_screening/na2co3_yield.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\to86hug\Desktop\Berechnungen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\to86hug\Desktop\two_photon_kinetics_parent\two_photon_kinetics\experimental_data\irradiations\additives\bases_screening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F50C117-6220-46BE-A08F-B789093A7EA2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9CABA4-4B0D-4E90-A913-357A4B132458}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{41A491FD-4B9E-374A-A7E5-31AA742B0AD0}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13305" xr2:uid="{41A491FD-4B9E-374A-A7E5-31AA742B0AD0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>0 ppm</t>
   </si>
@@ -430,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55A565D9-697E-0E4A-8B54-161E002639E6}">
-  <dimension ref="B1:N93"/>
+  <dimension ref="B1:N95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -563,70 +563,92 @@
       <c r="I6" s="4"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C7" s="1"/>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="4">
+        <f>D5*(SUM($D$2:$H$2)/SUM($D5:$H5))</f>
+        <v>213413.99516550062</v>
+      </c>
+      <c r="E7" s="4">
+        <f t="shared" ref="E7:I7" si="2">E5*(SUM($D$2:$H$2)/SUM($D5:$H5))</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <f t="shared" si="2"/>
+        <v>1723836.2165807062</v>
+      </c>
+      <c r="G7" s="4">
+        <f t="shared" si="2"/>
+        <v>471009.48537456529</v>
+      </c>
+      <c r="H7" s="4">
+        <f t="shared" si="2"/>
+        <v>83726.002879228239</v>
+      </c>
+      <c r="I7" s="4">
+        <f t="shared" si="2"/>
+        <v>9811430.8080157526</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C8" s="1"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C9" s="1"/>
+      <c r="D9" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I9" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C8" t="s">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="4">
-        <f>D5/$F$2</f>
-        <v>9.0739243319423693E-2</v>
-      </c>
-      <c r="E8" s="4">
-        <f>E5/$F$2</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="4">
-        <f>F5/$F$2</f>
-        <v>0.73293972018025089</v>
-      </c>
-      <c r="G8" s="4">
-        <f>G5/$F$2</f>
-        <v>0.20026355003576721</v>
-      </c>
-      <c r="H8" s="4">
-        <f>H5/$F$2</f>
-        <v>3.5598575161528055E-2</v>
-      </c>
-      <c r="I8" s="4">
-        <f>1-SUM(D8:H8)</f>
-        <v>-5.9541088696969835E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="D10" s="4">
+        <f>D7/$F$2</f>
+        <v>8.5640136364145511E-2</v>
+      </c>
+      <c r="E10" s="4">
+        <f t="shared" ref="E10:H10" si="3">E7/$F$2</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <f t="shared" si="3"/>
+        <v>0.69175205001405349</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" si="3"/>
+        <v>0.18900970634565248</v>
+      </c>
+      <c r="H10" s="4">
+        <f t="shared" si="3"/>
+        <v>3.3598107276148585E-2</v>
+      </c>
+      <c r="I10" s="4">
+        <f>1-SUM(D10:H10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D14" s="4"/>
@@ -645,7 +667,6 @@
       <c r="I15" s="4"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C16" s="1"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -654,7 +675,6 @@
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C17" s="1"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
@@ -663,6 +683,7 @@
       <c r="I17" s="4"/>
     </row>
     <row r="18" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C18" s="1"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
@@ -670,11 +691,22 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="57" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N57" s="2"/>
-    </row>
-    <row r="58" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N58" s="2"/>
+    <row r="19" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C19" s="1"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+    </row>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
     </row>
     <row r="59" spans="14:14" x14ac:dyDescent="0.25">
       <c r="N59" s="2"/>
@@ -779,7 +811,13 @@
       <c r="N92" s="2"/>
     </row>
     <row r="93" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N93" s="3"/>
+      <c r="N93" s="2"/>
+    </row>
+    <row r="94" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N94" s="2"/>
+    </row>
+    <row r="95" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N95" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>